<commit_message>
Update LocalizedBean type and refresh localization Excel files
</commit_message>
<xml_diff>
--- a/Templates~/Config/Excels/L10n/LocalizedAudio.xlsx
+++ b/Templates~/Config/Excels/L10n/LocalizedAudio.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Workspace\Unity\Project Abyss\Config\Datas\L10n\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Workspace\Unity\Game Dev Tools\Config\Excels\L10n\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A3CC4D7-D78C-4909-B631-C68D35A498FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85A66C44-ADA5-481B-A1D1-CE6AD96C86D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5040" yWindow="4755" windowWidth="28800" windowHeight="14820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4980" yWindow="4980" windowWidth="28815" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -142,11 +142,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>L10n.LocalizedAudioBean</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>res</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>L10n.LocalizedBean</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -576,7 +576,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D1" s="6"/>
     </row>
@@ -588,7 +588,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="6"/>
     </row>

</xml_diff>